<commit_message>
refactor: rename "member" to "student" across the codebase
- Updated test files to reflect the change from "member" to "student" in naming conventions and functionality.
- Renamed relevant variables, functions, and comments to ensure consistency.
- Adjusted database schema and SQL functions to replace "member" with "student" in roles, tables, and related entities.
- Modified authentication fixtures to accommodate the new "student" role.
</commit_message>
<xml_diff>
--- a/dummy-murid-sman70.xlsx
+++ b/dummy-murid-sman70.xlsx
@@ -398,20 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L6"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="36.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="24.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,7 +410,7 @@
         <v>password</v>
       </c>
       <c r="D1" t="str">
-        <v>tipe_member</v>
+        <v>tipe_student</v>
       </c>
       <c r="E1" t="str">
         <v>tanggal_lahir</v>

</xml_diff>